<commit_message>
Enhance HPT data collection and dashboard filtering
</commit_message>
<xml_diff>
--- a/backend/data/facility_master.xlsx
+++ b/backend/data/facility_master.xlsx
@@ -5,7 +5,7 @@
   <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Grace\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Grace\Documents\Nakuru County HPT\backend\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -8233,6 +8233,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:Q812"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="13.26953125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A1" t="s">

</xml_diff>